<commit_message>
Ajustes en salida_sap, estilos y planilla de modelos de maquinarias
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/Unidades/plantilla_modelos_maquinarias.xlsx
+++ b/data/reference/Unidades/plantilla_modelos_maquinarias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tattersall-my.sharepoint.com/personal/sherrera_tattersall_cl/Documents/Escritorio/FACU/INPUTS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{74B0ED40-AC33-4667-B411-C74549FB24E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CD3B6AD-362A-42CC-90FB-26B8407B8936}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{74B0ED40-AC33-4667-B411-C74549FB24E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8B8BB38-5C5F-4EF8-960A-A1211B1FA4BF}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="2025" windowWidth="20730" windowHeight="11040" tabRatio="790" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INPUT" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2041,9 +2041,6 @@
     <t>GRUA HORQUILLA</t>
   </si>
   <si>
-    <t>GRUA HOR</t>
-  </si>
-  <si>
     <t>GRUA PORTACONTENEDOR</t>
   </si>
   <si>
@@ -2060,6 +2057,9 @@
   </si>
   <si>
     <t>MANTELESC</t>
+  </si>
+  <si>
+    <t>GRUA-HOR</t>
   </si>
 </sst>
 </file>
@@ -2360,12 +2360,12 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6557,7 +6557,7 @@
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="3" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="3" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="3" customWidth="1"/>
@@ -6599,7 +6599,7 @@
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="V2" s="43" t="s">
+      <c r="V2" s="40" t="s">
         <v>16</v>
       </c>
       <c r="W2" s="41"/>
@@ -6607,7 +6607,7 @@
       <c r="Z2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="AE2" s="43" t="s">
+      <c r="AE2" s="40" t="s">
         <v>18</v>
       </c>
       <c r="AF2" s="41"/>
@@ -7139,7 +7139,7 @@
         <v>174</v>
       </c>
       <c r="S13" s="29" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="V13" s="31" t="s">
         <v>164</v>
@@ -7226,12 +7226,12 @@
         <v>196</v>
       </c>
       <c r="S16" s="29" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="V16" s="31"/>
       <c r="W16" s="31"/>
       <c r="X16" s="29"/>
-      <c r="Z16" s="40" t="s">
+      <c r="Z16" s="42" t="s">
         <v>186</v>
       </c>
       <c r="AA16" s="41"/>
@@ -7257,7 +7257,7 @@
       <c r="V17" s="31"/>
       <c r="W17" s="31"/>
       <c r="X17" s="29"/>
-      <c r="Z17" s="40" t="s">
+      <c r="Z17" s="42" t="s">
         <v>191</v>
       </c>
       <c r="AA17" s="41"/>
@@ -7279,7 +7279,7 @@
       <c r="V18" s="31"/>
       <c r="W18" s="31"/>
       <c r="X18" s="29"/>
-      <c r="Z18" s="42" t="s">
+      <c r="Z18" s="43" t="s">
         <v>194</v>
       </c>
       <c r="AA18" s="41"/>
@@ -7328,7 +7328,7 @@
         <v>657</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="S21" s="29" t="s">
         <v>657</v>
@@ -7336,7 +7336,7 @@
       <c r="V21" s="31"/>
       <c r="W21" s="31"/>
       <c r="X21" s="29"/>
-      <c r="Z21" s="40" t="s">
+      <c r="Z21" s="42" t="s">
         <v>202</v>
       </c>
       <c r="AA21" s="41"/>
@@ -7353,12 +7353,12 @@
         <v>117</v>
       </c>
       <c r="S22" s="29" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="V22" s="31"/>
       <c r="W22" s="31"/>
       <c r="X22" s="29"/>
-      <c r="Z22" s="40" t="s">
+      <c r="Z22" s="42" t="s">
         <v>205</v>
       </c>
       <c r="AA22" s="41"/>
@@ -7378,7 +7378,7 @@
       <c r="V23" s="31"/>
       <c r="W23" s="31"/>
       <c r="X23" s="29"/>
-      <c r="Z23" s="40" t="s">
+      <c r="Z23" s="42" t="s">
         <v>208</v>
       </c>
       <c r="AA23" s="41"/>
@@ -7398,7 +7398,7 @@
       <c r="V24" s="31"/>
       <c r="W24" s="31"/>
       <c r="X24" s="29"/>
-      <c r="Z24" s="40" t="s">
+      <c r="Z24" s="42" t="s">
         <v>209</v>
       </c>
       <c r="AA24" s="41"/>
@@ -7409,16 +7409,16 @@
     </row>
     <row r="25" spans="7:32" x14ac:dyDescent="0.25">
       <c r="G25" s="36" t="s">
+        <v>658</v>
+      </c>
+      <c r="H25" s="36" t="s">
         <v>659</v>
-      </c>
-      <c r="H25" s="36" t="s">
-        <v>660</v>
       </c>
       <c r="S25" s="29"/>
       <c r="V25" s="31"/>
       <c r="W25" s="31"/>
       <c r="X25" s="29"/>
-      <c r="Z25" s="40" t="s">
+      <c r="Z25" s="42" t="s">
         <v>210</v>
       </c>
       <c r="AA25" s="41"/>
@@ -7429,16 +7429,16 @@
     </row>
     <row r="26" spans="7:32" x14ac:dyDescent="0.25">
       <c r="G26" s="36" t="s">
+        <v>660</v>
+      </c>
+      <c r="H26" s="36" t="s">
         <v>661</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>662</v>
       </c>
       <c r="S26" s="29"/>
       <c r="V26" s="31"/>
       <c r="W26" s="31"/>
       <c r="X26" s="29"/>
-      <c r="Z26" s="40" t="s">
+      <c r="Z26" s="42" t="s">
         <v>211</v>
       </c>
       <c r="AA26" s="41"/>
@@ -7449,16 +7449,16 @@
     </row>
     <row r="27" spans="7:32" x14ac:dyDescent="0.25">
       <c r="G27" s="36" t="s">
+        <v>662</v>
+      </c>
+      <c r="H27" s="36" t="s">
         <v>663</v>
-      </c>
-      <c r="H27" s="36" t="s">
-        <v>664</v>
       </c>
       <c r="S27" s="29"/>
       <c r="V27" s="31"/>
       <c r="W27" s="31"/>
       <c r="X27" s="29"/>
-      <c r="Z27" s="40" t="s">
+      <c r="Z27" s="42" t="s">
         <v>212</v>
       </c>
       <c r="AA27" s="41"/>
@@ -7544,20 +7544,20 @@
       <c r="AF40" s="31"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" sort="0" autoFilter="0"/>
+  <sheetProtection sort="0" autoFilter="0"/>
   <mergeCells count="12">
+    <mergeCell ref="Z27:AC27"/>
+    <mergeCell ref="Z22:AC22"/>
+    <mergeCell ref="Z26:AC26"/>
+    <mergeCell ref="Z17:AC17"/>
+    <mergeCell ref="Z18:AC18"/>
+    <mergeCell ref="Z21:AC21"/>
     <mergeCell ref="AE2:AF2"/>
     <mergeCell ref="Z24:AC24"/>
     <mergeCell ref="Z16:AC16"/>
     <mergeCell ref="Z25:AC25"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="Z23:AC23"/>
-    <mergeCell ref="Z27:AC27"/>
-    <mergeCell ref="Z22:AC22"/>
-    <mergeCell ref="Z26:AC26"/>
-    <mergeCell ref="Z17:AC17"/>
-    <mergeCell ref="Z18:AC18"/>
-    <mergeCell ref="Z21:AC21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>